<commit_message>
Added new question type
Counter type is about to completely working
"Show right answers" and deselection aint working
</commit_message>
<xml_diff>
--- a/Assets/Quiz Template/Example/Sheets/MegaQuiz.xlsx
+++ b/Assets/Quiz Template/Example/Sheets/MegaQuiz.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unity\Projects\Mega-Quiz\Assets\Quiz Template\Example\Sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Unity\Projects\Quiz-Template\Assets\Quiz Template\Example\Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C02B56-5A76-4A44-B2DE-31270D6DB494}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CC8FFE-8D0B-4867-BB56-B890B18FA609}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="132">
   <si>
     <t>Тип вопроса</t>
   </si>
@@ -392,9 +392,6 @@
     <t>Вопрос</t>
   </si>
   <si>
-    <t>Неправильный ответ 4</t>
-  </si>
-  <si>
     <t>2+3</t>
   </si>
   <si>
@@ -408,6 +405,18 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Выбери цифры по порядку</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>4</t>
   </si>
 </sst>
 </file>
@@ -993,6 +1002,50 @@
     </xdr:pic>
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>347502</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>195089</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Рисунок 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30713175-85A1-44CF-BEE8-319985FE6A0D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2533650" y="1143000"/>
+          <a:ext cx="347502" cy="195089"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2884,16 +2937,14 @@
       <c r="G1" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="23" t="s">
-        <v>123</v>
-      </c>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>127</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>128</v>
       </c>
       <c r="C2" s="24"/>
       <c r="D2" s="26">
@@ -2908,16 +2959,14 @@
       <c r="G2" s="26">
         <v>1</v>
       </c>
-      <c r="H2" s="26">
-        <v>-999</v>
-      </c>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C3" s="24"/>
       <c r="D3" s="26">
@@ -2932,16 +2981,14 @@
       <c r="G3" s="26">
         <v>0</v>
       </c>
-      <c r="H3" s="26">
-        <v>-998</v>
-      </c>
+      <c r="H3" s="26"/>
     </row>
     <row r="4" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C4" s="24"/>
       <c r="D4" s="26">
@@ -2956,16 +3003,14 @@
       <c r="G4" s="26">
         <v>-1</v>
       </c>
-      <c r="H4" s="26">
-        <v>-997</v>
-      </c>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C5" s="24"/>
       <c r="D5" s="26">
@@ -2980,18 +3025,28 @@
       <c r="G5" s="26">
         <v>-2</v>
       </c>
-      <c r="H5" s="26">
-        <v>-996</v>
-      </c>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25"/>
-      <c r="B6" s="25"/>
+      <c r="A6" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>128</v>
+      </c>
       <c r="C6" s="24"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
+      <c r="D6" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="E6" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="F6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>131</v>
+      </c>
       <c r="H6" s="26"/>
     </row>
     <row r="7" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>